<commit_message>
Add final_2026.xlsx with initial data and structure
</commit_message>
<xml_diff>
--- a/final_2021.xlsx
+++ b/final_2021.xlsx
@@ -8,12 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Product_AMI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91752A58-8E94-42CA-8097-9D87AB5C2ADA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DECE86D8-E4C7-4AE9-ACD5-5E221AEC049B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{610C62FC-771F-46CD-9203-53674410F396}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="3" xr2:uid="{610C62FC-771F-46CD-9203-53674410F396}"/>
   </bookViews>
   <sheets>
     <sheet name="2" sheetId="1" r:id="rId1"/>
+    <sheet name="3" sheetId="2" r:id="rId2"/>
+    <sheet name="5" sheetId="3" r:id="rId3"/>
+    <sheet name="6" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,6 +36,44 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+  <si>
+    <t>งาน</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>ค่าปรับ</t>
+  </si>
+  <si>
+    <t>กำไรต่อล็อต</t>
+  </si>
+  <si>
+    <t>กำไรรวม</t>
+  </si>
+  <si>
+    <t>สุทธิ</t>
+  </si>
+  <si>
+    <t>ขาดทุนรวม</t>
+  </si>
+  <si>
+    <t>เวลารอบของทั้ง7</t>
+  </si>
+  <si>
+    <t>เวลาที่ใช้จริง</t>
+  </si>
+  <si>
+    <t>เวลาเหลืออ</t>
+  </si>
+  <si>
+    <t>sum</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -421,4 +462,573 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{531BED18-9951-40E1-B90D-75FA92659987}">
+  <dimension ref="A2:M14"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.09765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="4.8984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="3.8984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.8984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="3.8984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="4.8984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="3.8984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="4.8984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>4</v>
+      </c>
+      <c r="C2">
+        <v>10</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>9</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>6</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>5</v>
+      </c>
+      <c r="J2">
+        <v>7</v>
+      </c>
+      <c r="K2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>-4</v>
+      </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
+      <c r="D3">
+        <v>-1</v>
+      </c>
+      <c r="E3">
+        <v>4</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
+      <c r="G3">
+        <v>-1</v>
+      </c>
+      <c r="H3">
+        <v>-1</v>
+      </c>
+      <c r="I3">
+        <v>-1</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <f>IF(B3&gt;=0, 60*B3, 0)</f>
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <f t="shared" ref="C4:K4" si="0">IF(C3&gt;=0, 60*C3, 0)</f>
+        <v>240</v>
+      </c>
+      <c r="D4">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <f t="shared" si="0"/>
+        <v>240</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="0"/>
+        <v>240</v>
+      </c>
+      <c r="G4">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <f t="shared" si="0"/>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>100</v>
+      </c>
+      <c r="C5">
+        <v>125</v>
+      </c>
+      <c r="D5">
+        <v>80</v>
+      </c>
+      <c r="E5">
+        <v>175</v>
+      </c>
+      <c r="F5">
+        <v>70</v>
+      </c>
+      <c r="G5">
+        <v>110</v>
+      </c>
+      <c r="H5">
+        <v>45</v>
+      </c>
+      <c r="I5">
+        <v>60</v>
+      </c>
+      <c r="J5">
+        <v>200</v>
+      </c>
+      <c r="K5">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B6">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>10</v>
+      </c>
+      <c r="D6">
+        <v>7</v>
+      </c>
+      <c r="E6">
+        <v>9</v>
+      </c>
+      <c r="F6">
+        <v>5</v>
+      </c>
+      <c r="G6">
+        <v>5</v>
+      </c>
+      <c r="H6">
+        <v>4</v>
+      </c>
+      <c r="I6">
+        <v>10</v>
+      </c>
+      <c r="J6">
+        <v>6</v>
+      </c>
+      <c r="K6">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B7">
+        <f>B5*B6</f>
+        <v>800</v>
+      </c>
+      <c r="C7">
+        <f t="shared" ref="C7:K7" si="1">C5*C6</f>
+        <v>1250</v>
+      </c>
+      <c r="D7">
+        <f t="shared" si="1"/>
+        <v>560</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="1"/>
+        <v>1575</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="1"/>
+        <v>350</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="1"/>
+        <v>550</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="1"/>
+        <v>180</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="1"/>
+        <v>600</v>
+      </c>
+      <c r="J7">
+        <f t="shared" si="1"/>
+        <v>1200</v>
+      </c>
+      <c r="K7">
+        <f t="shared" si="1"/>
+        <v>640</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8">
+        <f>SUM(B7:K7)</f>
+        <v>7705</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9">
+        <f>SUM(B4:K4)</f>
+        <v>840</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10">
+        <f>B8-B9</f>
+        <v>6865</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B12">
+        <v>70</v>
+      </c>
+      <c r="C12">
+        <v>45</v>
+      </c>
+      <c r="D12">
+        <v>80</v>
+      </c>
+      <c r="E12">
+        <v>100</v>
+      </c>
+      <c r="F12">
+        <v>60</v>
+      </c>
+      <c r="G12">
+        <v>110</v>
+      </c>
+      <c r="H12">
+        <v>200</v>
+      </c>
+      <c r="I12">
+        <v>80</v>
+      </c>
+      <c r="J12">
+        <v>175</v>
+      </c>
+      <c r="K12">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B13">
+        <v>5</v>
+      </c>
+      <c r="C13">
+        <v>4</v>
+      </c>
+      <c r="D13">
+        <v>7</v>
+      </c>
+      <c r="E13">
+        <v>8</v>
+      </c>
+      <c r="F13">
+        <v>10</v>
+      </c>
+      <c r="G13">
+        <v>5</v>
+      </c>
+      <c r="H13">
+        <v>6</v>
+      </c>
+      <c r="I13">
+        <v>8</v>
+      </c>
+      <c r="J13">
+        <v>9</v>
+      </c>
+      <c r="K13">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B14">
+        <f>B12*B13</f>
+        <v>350</v>
+      </c>
+      <c r="C14">
+        <f t="shared" ref="C14:K14" si="2">C12*C13</f>
+        <v>180</v>
+      </c>
+      <c r="D14">
+        <f t="shared" si="2"/>
+        <v>560</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="2"/>
+        <v>800</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="2"/>
+        <v>600</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="2"/>
+        <v>550</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="2"/>
+        <v>1200</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="2"/>
+        <v>640</v>
+      </c>
+      <c r="J14">
+        <f t="shared" si="2"/>
+        <v>1575</v>
+      </c>
+      <c r="K14">
+        <f t="shared" si="2"/>
+        <v>1250</v>
+      </c>
+      <c r="L14" t="s">
+        <v>10</v>
+      </c>
+      <c r="M14">
+        <f>SUM(B14:K14)</f>
+        <v>7705</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4A78029-AB33-4626-A3AB-775E9281FB29}">
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1">
+        <v>44</v>
+      </c>
+      <c r="B1">
+        <v>44</v>
+      </c>
+      <c r="C1">
+        <v>44</v>
+      </c>
+      <c r="D1">
+        <v>44</v>
+      </c>
+      <c r="E1">
+        <v>44</v>
+      </c>
+      <c r="F1">
+        <v>44</v>
+      </c>
+      <c r="G1">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>44</v>
+      </c>
+      <c r="B2">
+        <v>43</v>
+      </c>
+      <c r="C2">
+        <v>44</v>
+      </c>
+      <c r="D2">
+        <v>44</v>
+      </c>
+      <c r="E2">
+        <v>44</v>
+      </c>
+      <c r="F2">
+        <v>41</v>
+      </c>
+      <c r="G2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <f>A1-A2</f>
+        <v>0</v>
+      </c>
+      <c r="B3">
+        <f>B1-B2</f>
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <f t="shared" ref="C3:G3" si="0">C1-C2</f>
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="G3">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <f>7*44</f>
+        <v>308</v>
+      </c>
+      <c r="B5">
+        <f>SUM(A2:G2)</f>
+        <v>295</v>
+      </c>
+      <c r="C5">
+        <f>A5-B5</f>
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93FE562C-5979-4B11-B614-57D103540808}">
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B1">
+        <v>0.5</v>
+      </c>
+      <c r="C1">
+        <v>0.6</v>
+      </c>
+      <c r="D1">
+        <v>2.9</v>
+      </c>
+      <c r="E1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <f>A1^2</f>
+        <v>4.8400000000000007</v>
+      </c>
+      <c r="B2">
+        <f t="shared" ref="B2:E2" si="0">B1^2</f>
+        <v>0.25</v>
+      </c>
+      <c r="C2">
+        <f t="shared" si="0"/>
+        <v>0.36</v>
+      </c>
+      <c r="D2">
+        <f t="shared" si="0"/>
+        <v>8.41</v>
+      </c>
+      <c r="E2">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <f>SQRT(SUM(A2:E2))</f>
+        <v>4.2261093218230874</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <f>_xlfn.NORM.INV(0.99,108,4.266)</f>
+        <v>117.92420003065823</v>
+      </c>
+      <c r="B6">
+        <f>(A6-108)/4.226</f>
+        <v>2.3483672576096137</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <f>_xlfn.NORM.DIST(A6,108, 4.226,TRUE)</f>
+        <v>0.99057204053289316</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>